<commit_message>
Enhance OPF results export and sensitivity analysis
- Added aggregation of AC, DC, and port losses in `export_results` function, including summary DataFrame for Excel export.
- Improved error handling in `run_sensitivity` function to capture optimization failures and log relevant details.
- Modified `run_optimization` function to allow optional suppression of exceptions on solver failure, returning instance with status metadata instead.
- Introduced new module `slack_tree.py` for slack-tree enumeration and analysis, including graph construction, spanning tree enumeration, port role assignment, validation, and interactive plotting.
- Implemented comprehensive slack-tree analysis pipeline in `run_slack_tree_analysis`, integrating OPF solving and results collection.
</commit_message>
<xml_diff>
--- a/data/examples/6PR-setup.xlsx
+++ b/data/examples/6PR-setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Google Drive\PycharmProjects\prg-opf\data\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6702E51F-53C2-4B87-B5BC-E676E07559B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EE22FA-D48C-43D7-854C-6AD8133C6322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="5400" windowWidth="14400" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Routers" sheetId="1" r:id="rId1"/>
@@ -515,13 +515,7 @@
         <v>8</v>
       </c>
       <c r="D2">
-        <v>10000</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -535,13 +529,7 @@
         <v>9</v>
       </c>
       <c r="D3">
-        <v>10000</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -555,13 +543,7 @@
         <v>9</v>
       </c>
       <c r="D4">
-        <v>10000</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -574,12 +556,6 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -591,12 +567,6 @@
       <c r="C6" t="s">
         <v>11</v>
       </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -609,18 +579,12 @@
         <v>12</v>
       </c>
       <c r="D7">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
         <v>0</v>
       </c>
     </row>
@@ -635,13 +599,7 @@
         <v>9</v>
       </c>
       <c r="D8">
-        <v>10000</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -655,18 +613,12 @@
         <v>12</v>
       </c>
       <c r="D9">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E9">
-        <v>-1</v>
+        <v>-0.1</v>
       </c>
       <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
         <v>0</v>
       </c>
     </row>
@@ -680,12 +632,6 @@
       <c r="C10" t="s">
         <v>11</v>
       </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -698,13 +644,7 @@
         <v>9</v>
       </c>
       <c r="D11">
-        <v>10000</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -718,18 +658,12 @@
         <v>12</v>
       </c>
       <c r="D12">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E12">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
         <v>0</v>
       </c>
     </row>
@@ -743,18 +677,6 @@
       <c r="C13" t="s">
         <v>10</v>
       </c>
-      <c r="E13">
-        <v>-4.1632999999999996</v>
-      </c>
-      <c r="F13">
-        <v>1.9400000000000001E-2</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -767,13 +689,7 @@
         <v>9</v>
       </c>
       <c r="D14">
-        <v>10000</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -787,18 +703,12 @@
         <v>12</v>
       </c>
       <c r="D15">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E15">
-        <v>-2</v>
+        <v>-0.2</v>
       </c>
       <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
         <v>0</v>
       </c>
     </row>
@@ -812,14 +722,8 @@
       <c r="C16" t="s">
         <v>11</v>
       </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>6</v>
       </c>
@@ -830,16 +734,10 @@
         <v>9</v>
       </c>
       <c r="D17">
-        <v>10000</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>6</v>
       </c>
@@ -850,22 +748,16 @@
         <v>12</v>
       </c>
       <c r="D18">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="E18">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6</v>
       </c>
@@ -874,12 +766,6 @@
       </c>
       <c r="C19" t="s">
         <v>11</v>
-      </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
-      <c r="H19">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -947,10 +833,10 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D2">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -964,10 +850,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D3">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E3">
         <v>100</v>
@@ -981,10 +867,10 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D4">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E4">
         <v>100</v>
@@ -998,10 +884,10 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D5">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -1015,10 +901,10 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D6">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -1032,10 +918,10 @@
         <v>15</v>
       </c>
       <c r="C7">
-        <v>17.82</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="D7">
-        <v>13.81</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="E7">
         <v>100</v>

</xml_diff>

<commit_message>
Add modified IEEE 9-bus system Excel file to examples directory
</commit_message>
<xml_diff>
--- a/data/examples/6PR-setup.xlsx
+++ b/data/examples/6PR-setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Google Drive\PycharmProjects\prg-opf\data\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EE22FA-D48C-43D7-854C-6AD8133C6322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967B3D9D-A29A-4925-B00E-DE3EC16C1975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="5400" windowWidth="14400" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Routers" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,19 @@
     <sheet name="DC Lines" sheetId="4" r:id="rId4"/>
     <sheet name="Parameters" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -554,7 +565,13 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>-1.03</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -675,7 +692,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -833,10 +850,10 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>0.48499999999999999</v>
+        <v>1.4550000000000001</v>
       </c>
       <c r="D2">
-        <v>0.78700000000000003</v>
+        <v>2.3610000000000002</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -901,10 +918,10 @@
         <v>11</v>
       </c>
       <c r="C6">
-        <v>0.48499999999999999</v>
+        <v>1.4550000000000001</v>
       </c>
       <c r="D6">
-        <v>0.78700000000000003</v>
+        <v>2.3610000000000002</v>
       </c>
       <c r="E6">
         <v>100</v>

</xml_diff>

<commit_message>
feat: enhance constraints and results handling for thermal limits and overloads
</commit_message>
<xml_diff>
--- a/data/examples/6PR-setup.xlsx
+++ b/data/examples/6PR-setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Google Drive\PycharmProjects\prg-opf\data\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967B3D9D-A29A-4925-B00E-DE3EC16C1975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95CA78D-122F-46B7-9B62-B92B86713E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10188" yWindow="5904" windowWidth="19200" windowHeight="12300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Routers" sheetId="1" r:id="rId1"/>
@@ -567,9 +567,6 @@
       <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="E5">
-        <v>-1.03</v>
-      </c>
       <c r="F5">
         <v>0</v>
       </c>
@@ -856,7 +853,7 @@
         <v>2.3610000000000002</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -873,7 +870,7 @@
         <v>0.78700000000000003</v>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -890,7 +887,7 @@
         <v>0.78700000000000003</v>
       </c>
       <c r="E4">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -907,7 +904,7 @@
         <v>0.78700000000000003</v>
       </c>
       <c r="E5">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -924,7 +921,7 @@
         <v>2.3610000000000002</v>
       </c>
       <c r="E6">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -941,7 +938,7 @@
         <v>0.78700000000000003</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>